<commit_message>
fix(inventory): correct sodium-ion module production name
Correct the copied LiS label on the sodium-ion module production exchange to match its existing SIB parent activity. Preserve its product and every quantity, including previously corrected sodium-ion capacity baselines. Document the identity-only scope in the existing activity comment.

Scope: existing supplemental workbook inventories only. Approved as item 5 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-SIB.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-SIB.xlsx
@@ -8987,8 +8987,12 @@
       <c r="A484" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B484" s="3" t="s">
-        <v>253</v>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED SODIUM-ION PRODUCTION-EXCHANGE IDENTITY, 2026-10-18. The parent activity is battery module production, for SiB battery, with output battery, SiB module. Correct only the copied LiS production-exchange name to match the SIB parent. Product, reference amount, cell fraction, all recipe coefficients and existing capacity normalization remain unchanged. This is an identity correction; no numerical system-metal effect or complete equipment coverage is established.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Taken from Wickerts et al. (2023). Prospective Life Cycle Assessment of Lithium-Sulfur Batteries for Stationary Energy Storage. ACS Sustainable Chemistry &amp; Engineering. Based on Ainsworth (2016), Peters and Weil (2017), Ellingsen et al. (2014) and adapted to SiB battery cells.</t>
+        </is>
       </c>
     </row>
     <row r="485" spans="1:11" x14ac:dyDescent="0.25">
@@ -9063,8 +9067,10 @@
       </c>
     </row>
     <row r="492" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A492" t="s">
-        <v>238</v>
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>battery module production, for SiB battery</t>
+        </is>
       </c>
       <c r="B492">
         <v>1</v>

</xml_diff>